<commit_message>
Configurar volumen persistente para datos
</commit_message>
<xml_diff>
--- a/data/adonai_data_completo.xlsx
+++ b/data/adonai_data_completo.xlsx
@@ -1179,7 +1179,6 @@
           <t>Donaciones USA</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>base</t>
@@ -1206,7 +1205,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="18.33203125" customWidth="1" min="3" max="3"/>
@@ -1383,6 +1382,47 @@
         <v>4999999.95</v>
       </c>
       <c r="I4" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>banco</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>egresos</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>1. Nómina</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Prestamos</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>fdsfsd</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>500000</v>
+      </c>
+      <c r="I5" t="inlineStr">
         <is>
           <t>admin</t>
         </is>
@@ -1453,7 +1493,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10019999.95</v>
+        <v>10519999.95</v>
       </c>
     </row>
     <row r="4">
@@ -1463,7 +1503,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-6019999.949999999</v>
+        <v>-6519999.949999999</v>
       </c>
     </row>
   </sheetData>
@@ -1617,10 +1657,10 @@
         <v>500000</v>
       </c>
       <c r="C6" t="n">
-        <v>4999999.95</v>
+        <v>5499999.95</v>
       </c>
       <c r="D6" t="n">
-        <v>-4499999.95</v>
+        <v>-4999999.95</v>
       </c>
     </row>
     <row r="7">
@@ -1724,7 +1764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1779,6 +1819,16 @@
         <v>3800</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-12</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>4500</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fixes 1-11 y funcionalidad de gestion de categorias
</commit_message>
<xml_diff>
--- a/data/adonai_data_completo.xlsx
+++ b/data/adonai_data_completo.xlsx
@@ -15,6 +15,8 @@
     <sheet name="Informe Mensual" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Configuracion" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="TRM" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Categorias" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Subcategorias" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -554,6 +556,2092 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>NombreEN</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ingreso</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Administrativo</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Administrative</t>
+        </is>
+      </c>
+      <c r="E2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ingreso</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Misión Institucional</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Institutional Mission</t>
+        </is>
+      </c>
+      <c r="E3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ingreso</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Unidad de Negocio</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Business Unit</t>
+        </is>
+      </c>
+      <c r="E4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ingreso</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Otros ingresos</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Other Income</t>
+        </is>
+      </c>
+      <c r="E5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>egreso</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1. Nómina</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1. Payroll</t>
+        </is>
+      </c>
+      <c r="E6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>egreso</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2. Colaboradoras Internas</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2. Internal Collaborators</t>
+        </is>
+      </c>
+      <c r="E7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>egreso</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>3. Proveedores</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>3. Suppliers</t>
+        </is>
+      </c>
+      <c r="E8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>egreso</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>4. Operacionales</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>4. Operational</t>
+        </is>
+      </c>
+      <c r="E9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>egreso</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>5. Redes Sociales</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>5. Social Media</t>
+        </is>
+      </c>
+      <c r="E10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>egreso</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>6. Material Publicitario</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>6. Advertising Material</t>
+        </is>
+      </c>
+      <c r="E11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>egreso</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>7. Trabajo de Campo</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>7. Field Work</t>
+        </is>
+      </c>
+      <c r="E12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>egreso</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>8. Otros Gastos</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>8. Other Expenses</t>
+        </is>
+      </c>
+      <c r="E13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>egreso</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>9. Misional Bebés</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>9. Missional Babies</t>
+        </is>
+      </c>
+      <c r="E14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>egreso</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>10. Misional Madres</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>10. Missional Mothers</t>
+        </is>
+      </c>
+      <c r="E15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>egreso</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>11. Otros</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>11. Otros</t>
+        </is>
+      </c>
+      <c r="E16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E80"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>CategoriaID</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>NombreEN</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Activo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Sostenimiento SRL</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>SRL Maintenance</t>
+        </is>
+      </c>
+      <c r="E2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Inversiones</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Investments</t>
+        </is>
+      </c>
+      <c r="E3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Donaciones locales</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Local Donations</t>
+        </is>
+      </c>
+      <c r="E4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Donaciones específicas locales</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Specific Local Donations</t>
+        </is>
+      </c>
+      <c r="E5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Donaciones USA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>USA Donations</t>
+        </is>
+      </c>
+      <c r="E6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Donaciones específicas USA</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Specific USA Donations</t>
+        </is>
+      </c>
+      <c r="E7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Donaciones ropa caja</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Clothing Donations</t>
+        </is>
+      </c>
+      <c r="E8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Jabón</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Soap</t>
+        </is>
+      </c>
+      <c r="E9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Otros ingresos</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Other Income</t>
+        </is>
+      </c>
+      <c r="E10" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="n">
+        <v>5</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Secretaria</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Secretary</t>
+        </is>
+      </c>
+      <c r="E11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Dirección General</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>General Direction</t>
+        </is>
+      </c>
+      <c r="E12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="n">
+        <v>5</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Seguridad Social</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Social Security</t>
+        </is>
+      </c>
+      <c r="E13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="n">
+        <v>5</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Prestaciones Sociales</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Social Benefits</t>
+        </is>
+      </c>
+      <c r="E14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Dotación</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Endowment</t>
+        </is>
+      </c>
+      <c r="E15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="n">
+        <v>5</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Prestamos</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Loans</t>
+        </is>
+      </c>
+      <c r="E16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="n">
+        <v>6</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Colaboradoras</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Collaborators</t>
+        </is>
+      </c>
+      <c r="E17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="n">
+        <v>7</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Dirección Misional</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Missional Direction</t>
+        </is>
+      </c>
+      <c r="E18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="n">
+        <v>7</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Administradora de redes sociales</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Social Media Admin</t>
+        </is>
+      </c>
+      <c r="E19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="n">
+        <v>7</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Servicios</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
+      <c r="E20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="n">
+        <v>7</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Honorarios</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Fees</t>
+        </is>
+      </c>
+      <c r="E21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="n">
+        <v>7</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Cuentas de cobro</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Bills</t>
+        </is>
+      </c>
+      <c r="E22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="n">
+        <v>8</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Renta</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Rent</t>
+        </is>
+      </c>
+      <c r="E23" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="n">
+        <v>8</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Servicios públicos</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Public Services</t>
+        </is>
+      </c>
+      <c r="E24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="n">
+        <v>8</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Internet</t>
+        </is>
+      </c>
+      <c r="E25" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="n">
+        <v>8</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Celular</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E26" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="n">
+        <v>8</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Compras insumos</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Supplies Purchases</t>
+        </is>
+      </c>
+      <c r="E27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="n">
+        <v>8</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Compras equipos de tecnología</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Tech Equipment Purchases</t>
+        </is>
+      </c>
+      <c r="E28" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="n">
+        <v>8</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Compras licencias</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Licenses Purchases</t>
+        </is>
+      </c>
+      <c r="E29" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="n">
+        <v>8</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Compras inmuebles</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Real Estate Purchases</t>
+        </is>
+      </c>
+      <c r="E30" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="n">
+        <v>8</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Obligaciones legales</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Legal Obligations</t>
+        </is>
+      </c>
+      <c r="E31" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Insumos cafetería</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Cafeteria Supplies</t>
+        </is>
+      </c>
+      <c r="E32" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="n">
+        <v>8</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Insumos de aseo</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Cleaning Supplies</t>
+        </is>
+      </c>
+      <c r="E33" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="n">
+        <v>8</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Insumos papelería</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Stationery Supplies</t>
+        </is>
+      </c>
+      <c r="E34" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="n">
+        <v>8</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Transporte urbano</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Urban Transport</t>
+        </is>
+      </c>
+      <c r="E35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="n">
+        <v>8</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Transporte colaboradores</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Collaborators Transport</t>
+        </is>
+      </c>
+      <c r="E36" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="n">
+        <v>8</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Parqueaderos</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Parking</t>
+        </is>
+      </c>
+      <c r="E37" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="n">
+        <v>8</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Gasolina</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Gasoline</t>
+        </is>
+      </c>
+      <c r="E38" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="n">
+        <v>8</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Reparaciones</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Repairs</t>
+        </is>
+      </c>
+      <c r="E39" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="n">
+        <v>8</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Mantenimientos</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Maintenance</t>
+        </is>
+      </c>
+      <c r="E40" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="n">
+        <v>8</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Reunión Junta</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Board Meeting</t>
+        </is>
+      </c>
+      <c r="E41" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="n">
+        <v>8</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Refrigerios colaboradores</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Collaborators Snacks</t>
+        </is>
+      </c>
+      <c r="E42" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="n">
+        <v>9</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="E43" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="n">
+        <v>9</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="E44" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="n">
+        <v>9</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="E45" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="n">
+        <v>9</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Página Web</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="E46" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="n">
+        <v>10</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Impresos</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Prints</t>
+        </is>
+      </c>
+      <c r="E47" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="n">
+        <v>10</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Botones</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Buttons</t>
+        </is>
+      </c>
+      <c r="E48" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="n">
+        <v>10</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Brochure</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Brochure</t>
+        </is>
+      </c>
+      <c r="E49" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="n">
+        <v>10</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Pendones</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Banners</t>
+        </is>
+      </c>
+      <c r="E50" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="n">
+        <v>10</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Alcancias</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Donation boxes</t>
+        </is>
+      </c>
+      <c r="E51" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="n">
+        <v>10</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Tarjetas de presentación</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Business Cards</t>
+        </is>
+      </c>
+      <c r="E52" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="n">
+        <v>10</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Cartas / Sobres con membrete</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Letters / Envelopes</t>
+        </is>
+      </c>
+      <c r="E53" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="n">
+        <v>10</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Audiovisuales</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Audiovisuals</t>
+        </is>
+      </c>
+      <c r="E54" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="n">
+        <v>11</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Reuniones externas</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>External Meetings</t>
+        </is>
+      </c>
+      <c r="E55" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="n">
+        <v>11</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Eventos locales</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Local Events</t>
+        </is>
+      </c>
+      <c r="E56" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="n">
+        <v>11</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Entrega publicidad</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Advertising Delivery</t>
+        </is>
+      </c>
+      <c r="E57" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="n">
+        <v>11</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Eventos fuera de medellín</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Events outside Medellin</t>
+        </is>
+      </c>
+      <c r="E58" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="n">
+        <v>12</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Gastos bancarios</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Bank Expenses</t>
+        </is>
+      </c>
+      <c r="E59" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="n">
+        <v>12</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Operacionales</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Operational</t>
+        </is>
+      </c>
+      <c r="E60" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" t="n">
+        <v>13</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Kit para el parto</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Delivery Kit</t>
+        </is>
+      </c>
+      <c r="E61" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" t="n">
+        <v>13</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Medicamentos</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Medicines</t>
+        </is>
+      </c>
+      <c r="E62" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" t="n">
+        <v>13</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Alimentos</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="E63" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" t="n">
+        <v>13</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Elementos básicos</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Basic Elements</t>
+        </is>
+      </c>
+      <c r="E64" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" t="n">
+        <v>13</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Cumpleaños</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Birthdays</t>
+        </is>
+      </c>
+      <c r="E65" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" t="n">
+        <v>13</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Jardín de la vida</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Garden of Life</t>
+        </is>
+      </c>
+      <c r="E66" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" t="n">
+        <v>13</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Hospitalizaciones</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Hospitalizations</t>
+        </is>
+      </c>
+      <c r="E67" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" t="n">
+        <v>14</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Kit para madres</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Mothers Kit</t>
+        </is>
+      </c>
+      <c r="E68" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" t="n">
+        <v>14</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Transporte</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="E69" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" t="n">
+        <v>14</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Alimentos</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Food</t>
+        </is>
+      </c>
+      <c r="E70" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" t="n">
+        <v>14</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Habitabilidad</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Housing</t>
+        </is>
+      </c>
+      <c r="E71" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" t="n">
+        <v>14</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Ayuda Humanitaria</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Humanitarian Aid</t>
+        </is>
+      </c>
+      <c r="E72" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" t="n">
+        <v>14</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Emprendimiento</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Entrepreneurship</t>
+        </is>
+      </c>
+      <c r="E73" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" t="n">
+        <v>14</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Obsequios</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Gifts</t>
+        </is>
+      </c>
+      <c r="E74" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" t="n">
+        <v>14</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Subsidio aliados</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Allies Subsidy</t>
+        </is>
+      </c>
+      <c r="E75" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" t="n">
+        <v>14</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Alianzas</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Alliances</t>
+        </is>
+      </c>
+      <c r="E76" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" t="n">
+        <v>15</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Otros</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E77" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" t="n">
+        <v>15</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Alianzas</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Alliances</t>
+        </is>
+      </c>
+      <c r="E78" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" t="n">
+        <v>15</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Apoyo Institucional</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Institutional Support</t>
+        </is>
+      </c>
+      <c r="E79" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" t="n">
+        <v>15</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Donaciones</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Donations</t>
+        </is>
+      </c>
+      <c r="E80" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -1413,7 +3501,6 @@
           <t>Prestamos</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>fdsfsd</t>

</xml_diff>